<commit_message>
M5 completado: mapa interactivo y visualizaciones
</commit_message>
<xml_diff>
--- a/resultados_akademia.xlsx
+++ b/resultados_akademia.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Ranking municipios" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Resumen por provincia" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Perfiles estratégicos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Guía de archivos" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -428,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q101"/>
+  <dimension ref="A1:R101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -517,6 +518,11 @@
           <t>perfil</t>
         </is>
       </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>perfil_corto</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -574,6 +580,11 @@
           <t>Zona premium — máxima solvencia</t>
         </is>
       </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -631,6 +642,11 @@
           <t>Zona premium — máxima solvencia</t>
         </is>
       </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -688,6 +704,11 @@
           <t>Zona premium — máxima solvencia</t>
         </is>
       </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -745,6 +766,11 @@
           <t>Zona premium — máxima solvencia</t>
         </is>
       </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -802,6 +828,11 @@
           <t>Zona premium — máxima solvencia</t>
         </is>
       </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -859,6 +890,11 @@
           <t>Zona premium — máxima solvencia</t>
         </is>
       </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -916,6 +952,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -973,6 +1014,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1030,6 +1076,11 @@
           <t>Gran ciudad — mercado masivo</t>
         </is>
       </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Gran ciudad</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1087,6 +1138,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1144,6 +1200,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1201,6 +1262,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1258,6 +1324,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1315,6 +1386,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1372,6 +1448,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1429,6 +1510,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1486,6 +1572,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1543,6 +1634,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1600,6 +1696,11 @@
           <t>Gran ciudad — mercado masivo</t>
         </is>
       </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Gran ciudad</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1657,6 +1758,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1714,6 +1820,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1771,6 +1882,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1828,6 +1944,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1885,6 +2007,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1940,6 +2068,12 @@
       <c r="Q26" t="inlineStr">
         <is>
           <t>Zona envejecida — solvencia ajustada</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
         </is>
       </c>
     </row>
@@ -1999,6 +2133,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2056,6 +2195,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2113,6 +2257,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2170,6 +2320,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2227,6 +2382,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2284,6 +2444,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2341,6 +2506,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2398,6 +2568,11 @@
           <t>Gran ciudad — mercado masivo</t>
         </is>
       </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Gran ciudad</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2455,6 +2630,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2510,6 +2690,11 @@
       <c r="Q36" t="inlineStr">
         <is>
           <t>Gran ciudad — mercado masivo</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Gran ciudad</t>
         </is>
       </c>
     </row>
@@ -2569,6 +2754,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2626,6 +2816,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2683,6 +2878,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2740,6 +2940,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2797,6 +3003,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2854,6 +3066,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2911,6 +3129,11 @@
           <t>Gran ciudad — mercado masivo</t>
         </is>
       </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Gran ciudad</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2968,6 +3191,11 @@
           <t>Gran ciudad — mercado masivo</t>
         </is>
       </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Gran ciudad</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -3025,6 +3253,11 @@
           <t>Gran ciudad — mercado masivo</t>
         </is>
       </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Gran ciudad</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -3082,6 +3315,11 @@
           <t>Gran ciudad — mercado masivo</t>
         </is>
       </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Gran ciudad</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -3139,6 +3377,11 @@
           <t>Gran ciudad — mercado masivo</t>
         </is>
       </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Gran ciudad</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -3196,6 +3439,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -3253,6 +3502,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -3310,6 +3564,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -3367,6 +3626,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -3424,6 +3688,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -3481,6 +3750,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -3538,6 +3812,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -3595,6 +3874,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -3652,6 +3936,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -3709,6 +3998,11 @@
           <t>Gran ciudad — mercado masivo</t>
         </is>
       </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>Gran ciudad</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -3766,6 +4060,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -3823,6 +4122,11 @@
           <t>Gran ciudad — mercado masivo</t>
         </is>
       </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>Gran ciudad</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -3880,6 +4184,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -3937,6 +4247,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -3994,6 +4309,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -4051,6 +4372,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -4108,6 +4435,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -4165,6 +4497,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -4222,6 +4560,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -4279,6 +4622,11 @@
           <t>Gran ciudad — mercado masivo</t>
         </is>
       </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>Gran ciudad</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -4336,6 +4684,11 @@
           <t>Gran ciudad — mercado masivo</t>
         </is>
       </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>Gran ciudad</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -4393,6 +4746,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -4450,6 +4808,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -4507,6 +4870,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -4564,6 +4932,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -4621,6 +4994,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -4678,6 +5056,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -4735,6 +5119,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -4792,6 +5181,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -4849,6 +5244,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -4906,6 +5306,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -4963,6 +5369,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -5020,6 +5432,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -5077,6 +5494,11 @@
           <t>Gran ciudad — mercado masivo</t>
         </is>
       </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>Gran ciudad</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -5134,6 +5556,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -5191,6 +5618,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -5248,6 +5680,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -5305,6 +5742,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -5362,6 +5805,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -5419,6 +5867,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -5476,6 +5930,11 @@
           <t>Gran ciudad — mercado masivo</t>
         </is>
       </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>Gran ciudad</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -5533,6 +5992,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -5590,6 +6055,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -5647,6 +6118,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -5704,6 +6180,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -5761,6 +6243,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -5818,6 +6305,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -5875,6 +6368,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -5932,6 +6430,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -5989,6 +6493,12 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -6046,6 +6556,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -6103,6 +6618,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -6160,6 +6680,11 @@
           <t>Municipio equilibrado — perfil estándar</t>
         </is>
       </c>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>Estándar</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -6215,6 +6740,12 @@
       <c r="Q101" t="inlineStr">
         <is>
           <t>Zona envejecida — solvencia ajustada</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>Solvencia
+ajustada</t>
         </is>
       </c>
     </row>
@@ -30230,4 +30761,114 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Archivo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Para qué sirve</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>mapa_top100.html</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Mapa interactivo — abrir en navegador, clicar en cada punto</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>grafico_perfiles.png</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Gráfico de barras con los 4 perfiles estratégicos — meter en slides</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>grafico_top20.png</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ranking visual del top 20 municipios — meter en slides</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>grafico_solvencia_mercado.png</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Scatter solvencia vs mercado — meter en slides</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>resultados_akademia.xlsx</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Excel con todas las pestañas de resultados</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>top100_con_clusters.csv</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Datos completos del top 100 con perfil asignado</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>dataset_maestro.csv</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Dataset central con todas las variables calculadas</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
M3 v2: Excel de resultados actualizado con 5 pestañas
</commit_message>
<xml_diff>
--- a/resultados_akademia.xlsx
+++ b/resultados_akademia.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X101"/>
+  <dimension ref="A1:W101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -548,11 +548,6 @@
           <t>perfil</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>perfil_corto</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -628,11 +623,6 @@
           <t>Zona premium — máxima solvencia</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -708,11 +698,6 @@
           <t>Zona premium — máxima solvencia</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -788,11 +773,6 @@
           <t>Zona premium — máxima solvencia</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -868,11 +848,6 @@
           <t>Zona premium — máxima solvencia</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -948,11 +923,6 @@
           <t>Gran ciudad — mercado masivo</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>Gran ciudad</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1028,12 +998,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1109,11 +1073,6 @@
           <t>Gran ciudad — mercado masivo</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>Gran ciudad</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1189,11 +1148,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X9" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1269,11 +1223,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X10" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1349,12 +1298,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X11" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1430,12 +1373,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X12" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1511,11 +1448,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X13" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1591,11 +1523,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X14" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1671,12 +1598,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1752,12 +1673,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X16" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1833,11 +1748,6 @@
           <t>Gran ciudad — mercado masivo</t>
         </is>
       </c>
-      <c r="X17" t="inlineStr">
-        <is>
-          <t>Gran ciudad</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1913,11 +1823,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X18" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1993,11 +1898,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X19" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -2073,12 +1973,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X20" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -2154,11 +2048,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X21" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2234,11 +2123,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X22" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2314,12 +2198,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X23" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2395,11 +2273,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X24" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2475,12 +2348,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X25" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2556,11 +2423,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X26" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2636,11 +2498,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X27" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2716,11 +2573,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X28" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2796,11 +2648,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X29" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2876,12 +2723,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X30" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2955,11 +2796,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X31" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -3035,12 +2871,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X32" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -3116,12 +2946,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X33" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -3197,11 +3021,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X34" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -3277,12 +3096,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X35" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -3358,12 +3171,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X36" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -3439,12 +3246,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X37" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -3520,11 +3321,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X38" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -3600,12 +3396,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X39" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -3681,12 +3471,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X40" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -3762,12 +3546,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X41" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -3843,12 +3621,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X42" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -3924,11 +3696,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X43" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -4004,12 +3771,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X44" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -4085,12 +3846,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X45" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -4166,11 +3921,6 @@
           <t>Gran ciudad — mercado masivo</t>
         </is>
       </c>
-      <c r="X46" t="inlineStr">
-        <is>
-          <t>Gran ciudad</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -4246,11 +3996,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X47" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -4326,11 +4071,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X48" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -4406,12 +4146,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X49" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -4487,12 +4221,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X50" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -4568,11 +4296,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X51" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -4648,12 +4371,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X52" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -4729,11 +4446,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X53" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -4809,11 +4521,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X54" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -4889,11 +4596,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X55" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -4969,12 +4671,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X56" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -5050,11 +4746,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X57" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -5130,11 +4821,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X58" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -5210,12 +4896,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X59" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -5291,12 +4971,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X60" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -5372,12 +5046,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X61" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -5453,12 +5121,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X62" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -5534,12 +5196,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X63" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -5615,12 +5271,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X64" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -5696,11 +5346,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X65" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -5776,11 +5421,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X66" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -5856,12 +5496,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X67" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -5937,11 +5571,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X68" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -6017,12 +5646,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X69" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -6098,12 +5721,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X70" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -6179,11 +5796,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X71" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -6259,12 +5871,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X72" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -6340,12 +5946,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X73" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -6421,12 +6021,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X74" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -6502,12 +6096,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X75" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -6583,12 +6171,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X76" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -6664,12 +6246,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X77" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -6745,11 +6321,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X78" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -6825,11 +6396,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X79" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -6905,12 +6471,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X80" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -6986,12 +6546,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X81" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -7067,12 +6621,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X82" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -7148,11 +6696,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X83" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -7228,11 +6771,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X84" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -7308,12 +6846,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X85" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -7389,12 +6921,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X86" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -7470,11 +6996,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X87" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -7550,12 +7071,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X88" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -7631,12 +7146,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X89" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -7712,12 +7221,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X90" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -7793,12 +7296,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X91" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -7874,12 +7371,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X92" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -7955,11 +7446,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X93" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -8035,12 +7521,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X94" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -8116,11 +7596,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X95" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -8196,11 +7671,6 @@
           <t>Ciudad media — mercado relevante</t>
         </is>
       </c>
-      <c r="X96" t="inlineStr">
-        <is>
-          <t>Ciudad media</t>
-        </is>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -8274,12 +7744,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X97" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -8355,12 +7819,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X98" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -8436,12 +7894,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X99" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -8517,12 +7969,6 @@
           <t>Zona envejecida — solvencia ajustada</t>
         </is>
       </c>
-      <c r="X100" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
-        </is>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -8596,12 +8042,6 @@
       <c r="W101" t="inlineStr">
         <is>
           <t>Zona envejecida — solvencia ajustada</t>
-        </is>
-      </c>
-      <c r="X101" t="inlineStr">
-        <is>
-          <t>Solvencia
-ajustada</t>
         </is>
       </c>
     </row>
@@ -8971,7 +8411,7 @@
         <v>40.41240833333333</v>
       </c>
       <c r="S5" t="n">
-        <v>-3.888334666666665</v>
+        <v>-3.888334666666666</v>
       </c>
       <c r="T5" t="n">
         <v>4</v>
@@ -8993,7 +8433,7 @@
         <v>51</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4847794023813705</v>
+        <v>0.4847794023813706</v>
       </c>
       <c r="F6" t="n">
         <v>0.5077566522111981</v>
@@ -9078,7 +8518,7 @@
         <v>319329</v>
       </c>
       <c r="L7" t="n">
-        <v>0.9142261290996812</v>
+        <v>0.9142261290996813</v>
       </c>
       <c r="M7" t="n">
         <v>39613</v>
@@ -9121,7 +8561,7 @@
         <v>1068</v>
       </c>
       <c r="E8" t="n">
-        <v>0.43823438740435</v>
+        <v>0.4382343874043501</v>
       </c>
       <c r="F8" t="n">
         <v>0.5008186096978743</v>
@@ -9185,7 +8625,7 @@
         <v>45</v>
       </c>
       <c r="E9" t="n">
-        <v>0.4300104378358091</v>
+        <v>0.4300104378358092</v>
       </c>
       <c r="F9" t="n">
         <v>0.4439702879247481</v>
@@ -9249,7 +8689,7 @@
         <v>5</v>
       </c>
       <c r="E10" t="n">
-        <v>0.4273114272024347</v>
+        <v>0.4273114272024348</v>
       </c>
       <c r="F10" t="n">
         <v>0.4316250920747843</v>
@@ -9517,7 +8957,7 @@
         <v>3141</v>
       </c>
       <c r="I14" t="n">
-        <v>6.056076162310792</v>
+        <v>6.056076162310791</v>
       </c>
       <c r="J14" t="n">
         <v>1.749123352635103</v>
@@ -9569,7 +9009,7 @@
         <v>5</v>
       </c>
       <c r="E15" t="n">
-        <v>0.419872088112816</v>
+        <v>0.4198720881128161</v>
       </c>
       <c r="F15" t="n">
         <v>0.4248811738237891</v>
@@ -9968,7 +9408,7 @@
         <v>10.7536513216607</v>
       </c>
       <c r="J21" t="n">
-        <v>1.662399414212096</v>
+        <v>1.662399414212095</v>
       </c>
       <c r="K21" t="n">
         <v>19881</v>
@@ -10081,10 +9521,10 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>0.4014445370661</v>
+        <v>0.4014445370661001</v>
       </c>
       <c r="F23" t="n">
-        <v>0.409363285577031</v>
+        <v>0.4093632855770311</v>
       </c>
       <c r="G23" t="n">
         <v>1609</v>
@@ -10145,10 +9585,10 @@
         <v>8</v>
       </c>
       <c r="E24" t="n">
-        <v>0.4005090199348843</v>
+        <v>0.4005090199348844</v>
       </c>
       <c r="F24" t="n">
-        <v>0.4113456095546476</v>
+        <v>0.4113456095546477</v>
       </c>
       <c r="G24" t="n">
         <v>1142</v>
@@ -10340,7 +9780,7 @@
         <v>0.3970367508766875</v>
       </c>
       <c r="F27" t="n">
-        <v>0.4219724242267962</v>
+        <v>0.4219724242267963</v>
       </c>
       <c r="G27" t="n">
         <v>5520</v>
@@ -10404,7 +9844,7 @@
         <v>0.3965893437364171</v>
       </c>
       <c r="F28" t="n">
-        <v>0.4247937846737621</v>
+        <v>0.4247937846737622</v>
       </c>
       <c r="G28" t="n">
         <v>19697</v>
@@ -10465,7 +9905,7 @@
         <v>45</v>
       </c>
       <c r="E29" t="n">
-        <v>0.395681280366926</v>
+        <v>0.3956812803669261</v>
       </c>
       <c r="F29" t="n">
         <v>0.4186525982358722</v>
@@ -10596,7 +10036,7 @@
         <v>0.3939259329009059</v>
       </c>
       <c r="F31" t="n">
-        <v>0.4096895019792347</v>
+        <v>0.4096895019792348</v>
       </c>
       <c r="G31" t="n">
         <v>7809</v>
@@ -10660,7 +10100,7 @@
         <v>0.3936927671285551</v>
       </c>
       <c r="F32" t="n">
-        <v>0.4054971899163352</v>
+        <v>0.4054971899163353</v>
       </c>
       <c r="G32" t="n">
         <v>15857</v>
@@ -10721,7 +10161,7 @@
         <v>15</v>
       </c>
       <c r="E33" t="n">
-        <v>0.3932994468335214</v>
+        <v>0.3932994468335215</v>
       </c>
       <c r="F33" t="n">
         <v>0.4138761207962848</v>
@@ -10916,7 +10356,7 @@
         <v>0.3901560043592153</v>
       </c>
       <c r="F36" t="n">
-        <v>0.4310573778138027</v>
+        <v>0.4310573778138028</v>
       </c>
       <c r="G36" t="n">
         <v>4943</v>
@@ -11108,7 +10548,7 @@
         <v>0.3885511492249665</v>
       </c>
       <c r="F39" t="n">
-        <v>0.4062963611076703</v>
+        <v>0.4062963611076704</v>
       </c>
       <c r="G39" t="n">
         <v>3649</v>
@@ -11169,7 +10609,7 @@
         <v>31</v>
       </c>
       <c r="E40" t="n">
-        <v>0.3881643550528166</v>
+        <v>0.3881643550528167</v>
       </c>
       <c r="F40" t="n">
         <v>0.4029524221910833</v>
@@ -11233,7 +10673,7 @@
         <v>17</v>
       </c>
       <c r="E41" t="n">
-        <v>0.3875510537389265</v>
+        <v>0.3875510537389266</v>
       </c>
       <c r="F41" t="n">
         <v>0.3978122287219664</v>
@@ -11309,7 +10749,7 @@
         <v>1064</v>
       </c>
       <c r="I42" t="n">
-        <v>9.035307829716205</v>
+        <v>9.035307829716203</v>
       </c>
       <c r="J42" t="n">
         <v>1.435204762679754</v>
@@ -11361,7 +10801,7 @@
         <v>9</v>
       </c>
       <c r="E43" t="n">
-        <v>0.3865025101492191</v>
+        <v>0.3865025101492192</v>
       </c>
       <c r="F43" t="n">
         <v>0.3994604562223356</v>
@@ -11492,7 +10932,7 @@
         <v>0.3852515745175681</v>
       </c>
       <c r="F45" t="n">
-        <v>0.3996727303529975</v>
+        <v>0.3996727303529976</v>
       </c>
       <c r="G45" t="n">
         <v>12052</v>
@@ -11510,7 +10950,7 @@
         <v>12048</v>
       </c>
       <c r="L45" t="n">
-        <v>0.9694076082655541</v>
+        <v>0.9694076082655539</v>
       </c>
       <c r="M45" t="n">
         <v>26874</v>
@@ -11684,7 +11124,7 @@
         <v>0.3840601728753373</v>
       </c>
       <c r="F48" t="n">
-        <v>0.4012579135344258</v>
+        <v>0.4012579135344259</v>
       </c>
       <c r="G48" t="n">
         <v>20439</v>
@@ -11748,7 +11188,7 @@
         <v>0.3828955112052963</v>
       </c>
       <c r="F49" t="n">
-        <v>0.3859991049433038</v>
+        <v>0.3859991049433039</v>
       </c>
       <c r="G49" t="n">
         <v>475</v>
@@ -12004,7 +11444,7 @@
         <v>0.3808434521491061</v>
       </c>
       <c r="F53" t="n">
-        <v>0.403672606152368</v>
+        <v>0.4036726061523681</v>
       </c>
       <c r="G53" t="n">
         <v>2915</v>
@@ -12065,7 +11505,7 @@
         <v>137</v>
       </c>
       <c r="E54" t="n">
-        <v>0.380376645082321</v>
+        <v>0.3803766450823211</v>
       </c>
       <c r="F54" t="n">
         <v>0.3996640849353248</v>
@@ -12132,7 +11572,7 @@
         <v>0.3794772647641941</v>
       </c>
       <c r="F55" t="n">
-        <v>0.3959979800998416</v>
+        <v>0.3959979800998417</v>
       </c>
       <c r="G55" t="n">
         <v>4037</v>
@@ -12156,7 +11596,7 @@
         <v>31823</v>
       </c>
       <c r="N55" t="n">
-        <v>1281.549999999999</v>
+        <v>1281.55</v>
       </c>
       <c r="O55" t="n">
         <v>1645.4</v>
@@ -12272,13 +11712,13 @@
         <v>10.46124360510631</v>
       </c>
       <c r="J57" t="n">
-        <v>1.831254807970086</v>
+        <v>1.831254807970087</v>
       </c>
       <c r="K57" t="n">
         <v>7910</v>
       </c>
       <c r="L57" t="n">
-        <v>0.9758774464963172</v>
+        <v>0.9758774464963171</v>
       </c>
       <c r="M57" t="n">
         <v>30555</v>
@@ -12385,7 +11825,7 @@
         <v>12</v>
       </c>
       <c r="E59" t="n">
-        <v>0.3764199619469969</v>
+        <v>0.376419961946997</v>
       </c>
       <c r="F59" t="n">
         <v>0.3879095256430624</v>
@@ -12449,7 +11889,7 @@
         <v>3</v>
       </c>
       <c r="E60" t="n">
-        <v>0.376375885271227</v>
+        <v>0.3763758852712271</v>
       </c>
       <c r="F60" t="n">
         <v>0.3802668306404175</v>
@@ -12577,10 +12017,10 @@
         <v>11</v>
       </c>
       <c r="E62" t="n">
-        <v>0.3746687258517215</v>
+        <v>0.3746687258517216</v>
       </c>
       <c r="F62" t="n">
-        <v>0.3849434188163882</v>
+        <v>0.3849434188163883</v>
       </c>
       <c r="G62" t="n">
         <v>907</v>
@@ -12662,7 +12102,7 @@
         <v>391</v>
       </c>
       <c r="L63" t="n">
-        <v>1.222414779226722</v>
+        <v>1.222414779226721</v>
       </c>
       <c r="M63" t="n">
         <v>48264</v>
@@ -12705,7 +12145,7 @@
         <v>4</v>
       </c>
       <c r="E64" t="n">
-        <v>0.3734745910803766</v>
+        <v>0.3734745910803767</v>
       </c>
       <c r="F64" t="n">
         <v>0.38443622659578</v>
@@ -12811,7 +12251,7 @@
         <v>40.68065216666667</v>
       </c>
       <c r="S65" t="n">
-        <v>-3.622887166666666</v>
+        <v>-3.622887166666667</v>
       </c>
       <c r="T65" t="n">
         <v>64</v>
@@ -12833,7 +12273,7 @@
         <v>9</v>
       </c>
       <c r="E66" t="n">
-        <v>0.3699041360218369</v>
+        <v>0.369904136021837</v>
       </c>
       <c r="F66" t="n">
         <v>0.3918231273859549</v>
@@ -12897,7 +12337,7 @@
         <v>3</v>
       </c>
       <c r="E67" t="n">
-        <v>0.3693278205467056</v>
+        <v>0.3693278205467057</v>
       </c>
       <c r="F67" t="n">
         <v>0.3750863904888986</v>
@@ -13092,7 +12532,7 @@
         <v>0.3644276061921603</v>
       </c>
       <c r="F70" t="n">
-        <v>0.3844585154316089</v>
+        <v>0.384458515431609</v>
       </c>
       <c r="G70" t="n">
         <v>5554</v>
@@ -13104,7 +12544,7 @@
         <v>4.491093050992502</v>
       </c>
       <c r="J70" t="n">
-        <v>1.762816364595052</v>
+        <v>1.762816364595053</v>
       </c>
       <c r="K70" t="n">
         <v>11419</v>
@@ -13153,7 +12593,7 @@
         <v>5</v>
       </c>
       <c r="E71" t="n">
-        <v>0.3636655230702408</v>
+        <v>0.3636655230702409</v>
       </c>
       <c r="F71" t="n">
         <v>0.3720566590275161</v>
@@ -13348,7 +12788,7 @@
         <v>0.3624715625854929</v>
       </c>
       <c r="F74" t="n">
-        <v>0.3668475111728306</v>
+        <v>0.3668475111728307</v>
       </c>
       <c r="G74" t="n">
         <v>651</v>
@@ -13494,7 +12934,7 @@
         <v>1004</v>
       </c>
       <c r="L76" t="n">
-        <v>1.959189395903754</v>
+        <v>1.959189395903755</v>
       </c>
       <c r="M76" t="n">
         <v>40819</v>
@@ -13665,10 +13105,10 @@
         <v>1</v>
       </c>
       <c r="E79" t="n">
-        <v>0.3589500026778491</v>
+        <v>0.3589500026778492</v>
       </c>
       <c r="F79" t="n">
-        <v>0.3589500026778491</v>
+        <v>0.3589500026778492</v>
       </c>
       <c r="G79" t="n">
         <v>64</v>
@@ -13729,7 +13169,7 @@
         <v>9</v>
       </c>
       <c r="E80" t="n">
-        <v>0.3583163611528683</v>
+        <v>0.3583163611528684</v>
       </c>
       <c r="F80" t="n">
         <v>0.3680223783093874</v>
@@ -13857,7 +13297,7 @@
         <v>37</v>
       </c>
       <c r="E82" t="n">
-        <v>0.3572370294333511</v>
+        <v>0.3572370294333512</v>
       </c>
       <c r="F82" t="n">
         <v>0.3693886593503816</v>
@@ -13985,10 +13425,10 @@
         <v>4</v>
       </c>
       <c r="E84" t="n">
-        <v>0.3564901408509341</v>
+        <v>0.3564901408509342</v>
       </c>
       <c r="F84" t="n">
-        <v>0.3659229801701282</v>
+        <v>0.3659229801701283</v>
       </c>
       <c r="G84" t="n">
         <v>864</v>
@@ -14006,7 +13446,7 @@
         <v>1058</v>
       </c>
       <c r="L84" t="n">
-        <v>1.163100634274087</v>
+        <v>1.163100634274088</v>
       </c>
       <c r="M84" t="n">
         <v>40239</v>
@@ -14177,7 +13617,7 @@
         <v>2</v>
       </c>
       <c r="E87" t="n">
-        <v>0.3558658475588367</v>
+        <v>0.3558658475588368</v>
       </c>
       <c r="F87" t="n">
         <v>0.3600030116439514</v>
@@ -14372,7 +13812,7 @@
         <v>0.35353956958039</v>
       </c>
       <c r="F90" t="n">
-        <v>0.3581746853543885</v>
+        <v>0.3581746853543886</v>
       </c>
       <c r="G90" t="n">
         <v>870</v>
@@ -14564,7 +14004,7 @@
         <v>0.3526744205811833</v>
       </c>
       <c r="F93" t="n">
-        <v>0.3639405362855737</v>
+        <v>0.3639405362855738</v>
       </c>
       <c r="G93" t="n">
         <v>952</v>
@@ -14628,7 +14068,7 @@
         <v>0.3526463906410703</v>
       </c>
       <c r="F94" t="n">
-        <v>0.3698353941668685</v>
+        <v>0.3698353941668686</v>
       </c>
       <c r="G94" t="n">
         <v>2251</v>
@@ -14692,7 +14132,7 @@
         <v>0.3525438283506304</v>
       </c>
       <c r="F95" t="n">
-        <v>0.3611846153372366</v>
+        <v>0.3611846153372367</v>
       </c>
       <c r="G95" t="n">
         <v>2049</v>
@@ -14701,7 +14141,7 @@
         <v>1253</v>
       </c>
       <c r="I95" t="n">
-        <v>9.830101557888099</v>
+        <v>9.830101557888101</v>
       </c>
       <c r="J95" t="n">
         <v>1.672165547340094</v>
@@ -14765,7 +14205,7 @@
         <v>272</v>
       </c>
       <c r="I96" t="n">
-        <v>9.685651153807749</v>
+        <v>9.685651153807747</v>
       </c>
       <c r="J96" t="n">
         <v>1.844155844155844</v>
@@ -14884,7 +14324,7 @@
         <v>0.3504909622986595</v>
       </c>
       <c r="F98" t="n">
-        <v>0.3958613088003835</v>
+        <v>0.3958613088003836</v>
       </c>
       <c r="G98" t="n">
         <v>84138</v>
@@ -15140,7 +14580,7 @@
         <v>0.3484387521769014</v>
       </c>
       <c r="F102" t="n">
-        <v>0.3535277087564429</v>
+        <v>0.353527708756443</v>
       </c>
       <c r="G102" t="n">
         <v>492</v>
@@ -15521,7 +14961,7 @@
         <v>3</v>
       </c>
       <c r="E108" t="n">
-        <v>0.347494206529801</v>
+        <v>0.3474942065298011</v>
       </c>
       <c r="F108" t="n">
         <v>0.35155729286413</v>
@@ -15606,7 +15046,7 @@
         <v>570</v>
       </c>
       <c r="L109" t="n">
-        <v>1.290249093897393</v>
+        <v>1.290249093897392</v>
       </c>
       <c r="M109" t="n">
         <v>36820</v>
@@ -15713,7 +15153,7 @@
         <v>8</v>
       </c>
       <c r="E111" t="n">
-        <v>0.3473161857320109</v>
+        <v>0.347316185732011</v>
       </c>
       <c r="F111" t="n">
         <v>0.3623751540608129</v>
@@ -15917,7 +15357,7 @@
         <v>283</v>
       </c>
       <c r="I114" t="n">
-        <v>7.420144885828749</v>
+        <v>7.42014488582875</v>
       </c>
       <c r="J114" t="n">
         <v>1.744852941176471</v>
@@ -15969,7 +15409,7 @@
         <v>5</v>
       </c>
       <c r="E115" t="n">
-        <v>0.3445387503718536</v>
+        <v>0.3445387503718537</v>
       </c>
       <c r="F115" t="n">
         <v>0.3528937734744636</v>
@@ -16072,7 +15512,7 @@
         <v>0</v>
       </c>
       <c r="R116" t="n">
-        <v>41.646723</v>
+        <v>41.64672299999999</v>
       </c>
       <c r="S116" t="n">
         <v>2.2246395</v>
@@ -16432,7 +15872,7 @@
         <v>6.602240457057126</v>
       </c>
       <c r="J122" t="n">
-        <v>1.787901702412741</v>
+        <v>1.787901702412742</v>
       </c>
       <c r="K122" t="n">
         <v>4009</v>
@@ -16481,10 +15921,10 @@
         <v>4</v>
       </c>
       <c r="E123" t="n">
-        <v>0.3429391711160174</v>
+        <v>0.3429391711160175</v>
       </c>
       <c r="F123" t="n">
-        <v>0.3440759140193893</v>
+        <v>0.3440759140193894</v>
       </c>
       <c r="G123" t="n">
         <v>538</v>
@@ -16566,7 +16006,7 @@
         <v>646</v>
       </c>
       <c r="L124" t="n">
-        <v>0.9733196521415316</v>
+        <v>0.9733196521415315</v>
       </c>
       <c r="M124" t="n">
         <v>31216</v>
@@ -16609,7 +16049,7 @@
         <v>5</v>
       </c>
       <c r="E125" t="n">
-        <v>0.3425745150456661</v>
+        <v>0.3425745150456662</v>
       </c>
       <c r="F125" t="n">
         <v>0.3557973654320494</v>
@@ -16740,7 +16180,7 @@
         <v>0.3419902483940355</v>
       </c>
       <c r="F127" t="n">
-        <v>0.3572916938146931</v>
+        <v>0.3572916938146932</v>
       </c>
       <c r="G127" t="n">
         <v>1002</v>
@@ -16801,10 +16241,10 @@
         <v>4</v>
       </c>
       <c r="E128" t="n">
-        <v>0.341430820854751</v>
+        <v>0.3414308208547511</v>
       </c>
       <c r="F128" t="n">
-        <v>0.3473677125697982</v>
+        <v>0.3473677125697983</v>
       </c>
       <c r="G128" t="n">
         <v>854</v>
@@ -16944,7 +16384,7 @@
         <v>13.05752970235189</v>
       </c>
       <c r="J130" t="n">
-        <v>1.703760406389884</v>
+        <v>1.703760406389883</v>
       </c>
       <c r="K130" t="n">
         <v>642</v>
@@ -16996,7 +16436,7 @@
         <v>0.3404375415268026</v>
       </c>
       <c r="F131" t="n">
-        <v>0.357158660100719</v>
+        <v>0.3571586601007191</v>
       </c>
       <c r="G131" t="n">
         <v>1059</v>
@@ -17014,7 +16454,7 @@
         <v>1600</v>
       </c>
       <c r="L131" t="n">
-        <v>1.5371317652149</v>
+        <v>1.537131765214899</v>
       </c>
       <c r="M131" t="n">
         <v>38612</v>
@@ -17072,13 +16512,13 @@
         <v>9.80337986995522</v>
       </c>
       <c r="J132" t="n">
-        <v>1.655468035167284</v>
+        <v>1.655468035167283</v>
       </c>
       <c r="K132" t="n">
         <v>699</v>
       </c>
       <c r="L132" t="n">
-        <v>1.349917106902032</v>
+        <v>1.349917106902031</v>
       </c>
       <c r="M132" t="n">
         <v>35778</v>
@@ -17249,7 +16689,7 @@
         <v>10</v>
       </c>
       <c r="E135" t="n">
-        <v>0.3397393918684744</v>
+        <v>0.3397393918684745</v>
       </c>
       <c r="F135" t="n">
         <v>0.3490196149426877</v>
@@ -17264,13 +16704,13 @@
         <v>8.025755109182287</v>
       </c>
       <c r="J135" t="n">
-        <v>1.834735224426881</v>
+        <v>1.834735224426882</v>
       </c>
       <c r="K135" t="n">
         <v>1640</v>
       </c>
       <c r="L135" t="n">
-        <v>1.064240131553314</v>
+        <v>1.064240131553315</v>
       </c>
       <c r="M135" t="n">
         <v>36853</v>
@@ -17313,7 +16753,7 @@
         <v>3</v>
       </c>
       <c r="E136" t="n">
-        <v>0.3395182775403216</v>
+        <v>0.3395182775403217</v>
       </c>
       <c r="F136" t="n">
         <v>0.3599042121433954</v>
@@ -17569,10 +17009,10 @@
         <v>1</v>
       </c>
       <c r="E140" t="n">
-        <v>0.3389043976403409</v>
+        <v>0.338904397640341</v>
       </c>
       <c r="F140" t="n">
-        <v>0.3389043976403409</v>
+        <v>0.338904397640341</v>
       </c>
       <c r="G140" t="n">
         <v>32</v>
@@ -17633,10 +17073,10 @@
         <v>1</v>
       </c>
       <c r="E141" t="n">
-        <v>0.3378514600335778</v>
+        <v>0.3378514600335779</v>
       </c>
       <c r="F141" t="n">
-        <v>0.3378514600335778</v>
+        <v>0.3378514600335779</v>
       </c>
       <c r="G141" t="n">
         <v>38</v>
@@ -17956,7 +17396,7 @@
         <v>0.3371538055353117</v>
       </c>
       <c r="F146" t="n">
-        <v>0.3598515295673787</v>
+        <v>0.3598515295673788</v>
       </c>
       <c r="G146" t="n">
         <v>45720</v>
@@ -17968,7 +17408,7 @@
         <v>13.70222885208217</v>
       </c>
       <c r="J146" t="n">
-        <v>2.18702816193344</v>
+        <v>2.187028161933439</v>
       </c>
       <c r="K146" t="n">
         <v>40724</v>
@@ -18084,7 +17524,7 @@
         <v>0.3369303914800811</v>
       </c>
       <c r="F148" t="n">
-        <v>0.3571938683639717</v>
+        <v>0.3571938683639718</v>
       </c>
       <c r="G148" t="n">
         <v>23273</v>
@@ -18093,7 +17533,7 @@
         <v>14540</v>
       </c>
       <c r="I148" t="n">
-        <v>13.06230010984514</v>
+        <v>13.06230010984515</v>
       </c>
       <c r="J148" t="n">
         <v>2.182128026570019</v>
@@ -18148,7 +17588,7 @@
         <v>0.3369069158961846</v>
       </c>
       <c r="F149" t="n">
-        <v>0.3587779566964302</v>
+        <v>0.3587779566964303</v>
       </c>
       <c r="G149" t="n">
         <v>5142</v>
@@ -18209,10 +17649,10 @@
         <v>4</v>
       </c>
       <c r="E150" t="n">
-        <v>0.3367665989826386</v>
+        <v>0.3367665989826387</v>
       </c>
       <c r="F150" t="n">
-        <v>0.3420782775355406</v>
+        <v>0.3420782775355407</v>
       </c>
       <c r="G150" t="n">
         <v>665</v>
@@ -18276,7 +17716,7 @@
         <v>0.3366713227769409</v>
       </c>
       <c r="F151" t="n">
-        <v>0.3413913198707802</v>
+        <v>0.3413913198707803</v>
       </c>
       <c r="G151" t="n">
         <v>526</v>
@@ -18340,7 +17780,7 @@
         <v>0.3366517169307946</v>
       </c>
       <c r="F152" t="n">
-        <v>0.3376971337683271</v>
+        <v>0.3376971337683272</v>
       </c>
       <c r="G152" t="n">
         <v>310</v>
@@ -18465,10 +17905,10 @@
         <v>1</v>
       </c>
       <c r="E154" t="n">
-        <v>0.3363803136276705</v>
+        <v>0.3363803136276706</v>
       </c>
       <c r="F154" t="n">
-        <v>0.3363803136276705</v>
+        <v>0.3363803136276706</v>
       </c>
       <c r="G154" t="n">
         <v>188</v>
@@ -18593,10 +18033,10 @@
         <v>1</v>
       </c>
       <c r="E156" t="n">
-        <v>0.3363593208801403</v>
+        <v>0.3363593208801404</v>
       </c>
       <c r="F156" t="n">
-        <v>0.3363593208801403</v>
+        <v>0.3363593208801404</v>
       </c>
       <c r="G156" t="n">
         <v>11</v>
@@ -18934,7 +18374,7 @@
         <v>1748</v>
       </c>
       <c r="L161" t="n">
-        <v>1.21101184361336</v>
+        <v>1.211011843613359</v>
       </c>
       <c r="M161" t="n">
         <v>35802</v>
@@ -19169,10 +18609,10 @@
         <v>7</v>
       </c>
       <c r="E165" t="n">
-        <v>0.3347382032169316</v>
+        <v>0.3347382032169317</v>
       </c>
       <c r="F165" t="n">
-        <v>0.3428594020778038</v>
+        <v>0.3428594020778039</v>
       </c>
       <c r="G165" t="n">
         <v>925</v>
@@ -19297,7 +18737,7 @@
         <v>3</v>
       </c>
       <c r="E167" t="n">
-        <v>0.3343240645604314</v>
+        <v>0.3343240645604315</v>
       </c>
       <c r="F167" t="n">
         <v>0.3394629336735995</v>
@@ -19745,7 +19185,7 @@
         <v>6</v>
       </c>
       <c r="E174" t="n">
-        <v>0.3336115272062382</v>
+        <v>0.3336115272062383</v>
       </c>
       <c r="F174" t="n">
         <v>0.3366760052169868</v>
@@ -20016,7 +19456,7 @@
         <v>7.098020391957707</v>
       </c>
       <c r="J178" t="n">
-        <v>1.584300132050556</v>
+        <v>1.584300132050557</v>
       </c>
       <c r="K178" t="n">
         <v>557</v>
@@ -20232,7 +19672,7 @@
         <v>0</v>
       </c>
       <c r="R181" t="n">
-        <v>41.5001935</v>
+        <v>41.50019349999999</v>
       </c>
       <c r="S181" t="n">
         <v>1.8107835</v>
@@ -20321,7 +19761,7 @@
         <v>10</v>
       </c>
       <c r="E183" t="n">
-        <v>0.3323461046215545</v>
+        <v>0.3323461046215546</v>
       </c>
       <c r="F183" t="n">
         <v>0.3436782720398054</v>
@@ -20388,7 +19828,7 @@
         <v>0.3322064970080352</v>
       </c>
       <c r="F184" t="n">
-        <v>0.3374800212773512</v>
+        <v>0.3374800212773513</v>
       </c>
       <c r="G184" t="n">
         <v>239</v>
@@ -20513,10 +19953,10 @@
         <v>5</v>
       </c>
       <c r="E186" t="n">
-        <v>0.3321529740105023</v>
+        <v>0.3321529740105024</v>
       </c>
       <c r="F186" t="n">
-        <v>0.3370399722029228</v>
+        <v>0.3370399722029229</v>
       </c>
       <c r="G186" t="n">
         <v>361</v>
@@ -20641,7 +20081,7 @@
         <v>14</v>
       </c>
       <c r="E188" t="n">
-        <v>0.3320182686599205</v>
+        <v>0.3320182686599206</v>
       </c>
       <c r="F188" t="n">
         <v>0.3507133388878987</v>
@@ -20781,7 +20221,7 @@
         <v>710</v>
       </c>
       <c r="I190" t="n">
-        <v>7.865038304036035</v>
+        <v>7.865038304036037</v>
       </c>
       <c r="J190" t="n">
         <v>1.461013641648754</v>
@@ -20790,7 +20230,7 @@
         <v>1529</v>
       </c>
       <c r="L190" t="n">
-        <v>1.225822603603632</v>
+        <v>1.225822603603631</v>
       </c>
       <c r="M190" t="n">
         <v>35735</v>
@@ -20833,7 +20273,7 @@
         <v>3</v>
       </c>
       <c r="E191" t="n">
-        <v>0.3314039591001554</v>
+        <v>0.3314039591001555</v>
       </c>
       <c r="F191" t="n">
         <v>0.3365561550999066</v>
@@ -20912,7 +20352,7 @@
         <v>8.953676983482755</v>
       </c>
       <c r="J192" t="n">
-        <v>1.8141777356406</v>
+        <v>1.814177735640599</v>
       </c>
       <c r="K192" t="n">
         <v>7299</v>
@@ -21238,7 +20678,7 @@
         <v>676</v>
       </c>
       <c r="L197" t="n">
-        <v>1.047571718748807</v>
+        <v>1.047571718748806</v>
       </c>
       <c r="M197" t="n">
         <v>31683</v>
@@ -21284,7 +20724,7 @@
         <v>0.330252210035711</v>
       </c>
       <c r="F198" t="n">
-        <v>0.3341488848573328</v>
+        <v>0.3341488848573329</v>
       </c>
       <c r="G198" t="n">
         <v>351</v>
@@ -21412,7 +20852,7 @@
         <v>0.3302155520851952</v>
       </c>
       <c r="F200" t="n">
-        <v>0.3428193247519909</v>
+        <v>0.342819324751991</v>
       </c>
       <c r="G200" t="n">
         <v>1073</v>
@@ -21473,10 +20913,10 @@
         <v>6</v>
       </c>
       <c r="E201" t="n">
-        <v>0.3301903660471358</v>
+        <v>0.3301903660471359</v>
       </c>
       <c r="F201" t="n">
-        <v>0.3335031463741962</v>
+        <v>0.3335031463741963</v>
       </c>
       <c r="G201" t="n">
         <v>636</v>
@@ -21537,10 +20977,10 @@
         <v>2</v>
       </c>
       <c r="E202" t="n">
-        <v>0.3301301662951726</v>
+        <v>0.3301301662951727</v>
       </c>
       <c r="F202" t="n">
-        <v>0.3305676266655823</v>
+        <v>0.3305676266655824</v>
       </c>
       <c r="G202" t="n">
         <v>384</v>
@@ -21558,7 +20998,7 @@
         <v>404</v>
       </c>
       <c r="L202" t="n">
-        <v>0.993269648284846</v>
+        <v>0.9932696482848459</v>
       </c>
       <c r="M202" t="n">
         <v>31361</v>
@@ -21665,7 +21105,7 @@
         <v>41</v>
       </c>
       <c r="E204" t="n">
-        <v>0.3299831200654829</v>
+        <v>0.329983120065483</v>
       </c>
       <c r="F204" t="n">
         <v>0.3498282146338849</v>
@@ -21707,7 +21147,7 @@
         <v>39.67150431707317</v>
       </c>
       <c r="S204" t="n">
-        <v>-0.2472086585365853</v>
+        <v>-0.2472086585365854</v>
       </c>
       <c r="T204" t="n">
         <v>203</v>
@@ -21857,10 +21297,10 @@
         <v>3</v>
       </c>
       <c r="E207" t="n">
-        <v>0.329699968051822</v>
+        <v>0.3296999680518221</v>
       </c>
       <c r="F207" t="n">
-        <v>0.335309120694591</v>
+        <v>0.3353091206945911</v>
       </c>
       <c r="G207" t="n">
         <v>558</v>
@@ -21921,7 +21361,7 @@
         <v>4</v>
       </c>
       <c r="E208" t="n">
-        <v>0.3296807485305449</v>
+        <v>0.329680748530545</v>
       </c>
       <c r="F208" t="n">
         <v>0.3347690163770282</v>
@@ -21988,7 +21428,7 @@
         <v>0.3296353943204953</v>
       </c>
       <c r="F209" t="n">
-        <v>0.3396426098913377</v>
+        <v>0.3396426098913378</v>
       </c>
       <c r="G209" t="n">
         <v>1800</v>
@@ -22049,10 +21489,10 @@
         <v>1</v>
       </c>
       <c r="E210" t="n">
-        <v>0.3295647809053258</v>
+        <v>0.3295647809053259</v>
       </c>
       <c r="F210" t="n">
-        <v>0.3295647809053258</v>
+        <v>0.3295647809053259</v>
       </c>
       <c r="G210" t="n">
         <v>273</v>
@@ -22244,7 +21684,7 @@
         <v>0.329220750345429</v>
       </c>
       <c r="F213" t="n">
-        <v>0.3328598224838199</v>
+        <v>0.33285982248382</v>
       </c>
       <c r="G213" t="n">
         <v>626</v>
@@ -22369,10 +21809,10 @@
         <v>1</v>
       </c>
       <c r="E215" t="n">
-        <v>0.3288520458387898</v>
+        <v>0.3288520458387899</v>
       </c>
       <c r="F215" t="n">
-        <v>0.3288520458387898</v>
+        <v>0.3288520458387899</v>
       </c>
       <c r="G215" t="n">
         <v>22</v>
@@ -22817,7 +22257,7 @@
         <v>4</v>
       </c>
       <c r="E222" t="n">
-        <v>0.3281578627481791</v>
+        <v>0.3281578627481792</v>
       </c>
       <c r="F222" t="n">
         <v>0.3483945112197996</v>
@@ -23021,7 +22461,7 @@
         <v>188</v>
       </c>
       <c r="I225" t="n">
-        <v>9.317843498537416</v>
+        <v>9.317843498537417</v>
       </c>
       <c r="J225" t="n">
         <v>1.487108013937282</v>
@@ -23085,7 +22525,7 @@
         <v>861</v>
       </c>
       <c r="I226" t="n">
-        <v>9.689084092686649</v>
+        <v>9.689084092686647</v>
       </c>
       <c r="J226" t="n">
         <v>1.876049117562184</v>
@@ -23393,10 +22833,10 @@
         <v>3</v>
       </c>
       <c r="E231" t="n">
-        <v>0.3260987262923089</v>
+        <v>0.326098726292309</v>
       </c>
       <c r="F231" t="n">
-        <v>0.3345181867520292</v>
+        <v>0.3345181867520293</v>
       </c>
       <c r="G231" t="n">
         <v>446</v>
@@ -23521,10 +22961,10 @@
         <v>1</v>
       </c>
       <c r="E233" t="n">
-        <v>0.3258861843347507</v>
+        <v>0.3258861843347508</v>
       </c>
       <c r="F233" t="n">
-        <v>0.3258861843347507</v>
+        <v>0.3258861843347508</v>
       </c>
       <c r="G233" t="n">
         <v>102</v>
@@ -23585,10 +23025,10 @@
         <v>4</v>
       </c>
       <c r="E234" t="n">
-        <v>0.3257486488970021</v>
+        <v>0.3257486488970022</v>
       </c>
       <c r="F234" t="n">
-        <v>0.3313379288951161</v>
+        <v>0.3313379288951162</v>
       </c>
       <c r="G234" t="n">
         <v>753</v>
@@ -23905,10 +23345,10 @@
         <v>1</v>
       </c>
       <c r="E239" t="n">
-        <v>0.3255640243350475</v>
+        <v>0.3255640243350476</v>
       </c>
       <c r="F239" t="n">
-        <v>0.3255640243350475</v>
+        <v>0.3255640243350476</v>
       </c>
       <c r="G239" t="n">
         <v>92</v>
@@ -24033,10 +23473,10 @@
         <v>1</v>
       </c>
       <c r="E241" t="n">
-        <v>0.3254302555153422</v>
+        <v>0.3254302555153423</v>
       </c>
       <c r="F241" t="n">
-        <v>0.3254302555153422</v>
+        <v>0.3254302555153423</v>
       </c>
       <c r="G241" t="n">
         <v>267</v>
@@ -24112,7 +23552,7 @@
         <v>12.08517876777488</v>
       </c>
       <c r="J242" t="n">
-        <v>2.19399906119057</v>
+        <v>2.193999061190571</v>
       </c>
       <c r="K242" t="n">
         <v>15372</v>
@@ -24417,10 +23857,10 @@
         <v>1</v>
       </c>
       <c r="E247" t="n">
-        <v>0.3250442398952365</v>
+        <v>0.3250442398952366</v>
       </c>
       <c r="F247" t="n">
-        <v>0.3250442398952365</v>
+        <v>0.3250442398952366</v>
       </c>
       <c r="G247" t="n">
         <v>193</v>
@@ -24609,7 +24049,7 @@
         <v>6</v>
       </c>
       <c r="E250" t="n">
-        <v>0.3246494190107556</v>
+        <v>0.3246494190107557</v>
       </c>
       <c r="F250" t="n">
         <v>0.3339422166650123</v>
@@ -24624,7 +24064,7 @@
         <v>14.05672251361634</v>
       </c>
       <c r="J250" t="n">
-        <v>1.82621140555351</v>
+        <v>1.826211405553511</v>
       </c>
       <c r="K250" t="n">
         <v>842</v>
@@ -24712,7 +24152,7 @@
         <v>0</v>
       </c>
       <c r="R251" t="n">
-        <v>41.62632163636364</v>
+        <v>41.62632163636363</v>
       </c>
       <c r="S251" t="n">
         <v>2.299966</v>
@@ -25581,7 +25021,7 @@
         <v>187</v>
       </c>
       <c r="I265" t="n">
-        <v>9.127212594191391</v>
+        <v>9.127212594191393</v>
       </c>
       <c r="J265" t="n">
         <v>1.588806660499537</v>
@@ -25675,7 +25115,7 @@
         <v>38.40051353846154</v>
       </c>
       <c r="S266" t="n">
-        <v>-0.4339552307692307</v>
+        <v>-0.4339552307692308</v>
       </c>
       <c r="T266" t="n">
         <v>265</v>
@@ -25697,10 +25137,10 @@
         <v>1</v>
       </c>
       <c r="E267" t="n">
-        <v>0.3230905431231859</v>
+        <v>0.323090543123186</v>
       </c>
       <c r="F267" t="n">
-        <v>0.3230905431231859</v>
+        <v>0.323090543123186</v>
       </c>
       <c r="G267" t="n">
         <v>18</v>
@@ -25889,10 +25329,10 @@
         <v>1</v>
       </c>
       <c r="E270" t="n">
-        <v>0.3228713337193747</v>
+        <v>0.3228713337193748</v>
       </c>
       <c r="F270" t="n">
-        <v>0.3228713337193747</v>
+        <v>0.3228713337193748</v>
       </c>
       <c r="G270" t="n">
         <v>77</v>
@@ -25953,7 +25393,7 @@
         <v>12</v>
       </c>
       <c r="E271" t="n">
-        <v>0.322806648431384</v>
+        <v>0.3228066484313841</v>
       </c>
       <c r="F271" t="n">
         <v>0.3360812302462473</v>
@@ -26209,10 +25649,10 @@
         <v>1</v>
       </c>
       <c r="E275" t="n">
-        <v>0.3222172051185519</v>
+        <v>0.322217205118552</v>
       </c>
       <c r="F275" t="n">
-        <v>0.3222172051185519</v>
+        <v>0.322217205118552</v>
       </c>
       <c r="G275" t="n">
         <v>27</v>
@@ -26465,10 +25905,10 @@
         <v>1</v>
       </c>
       <c r="E279" t="n">
-        <v>0.3217571277854826</v>
+        <v>0.3217571277854827</v>
       </c>
       <c r="F279" t="n">
-        <v>0.3217571277854826</v>
+        <v>0.3217571277854827</v>
       </c>
       <c r="G279" t="n">
         <v>31</v>
@@ -26532,7 +25972,7 @@
         <v>0.3217503126052968</v>
       </c>
       <c r="F280" t="n">
-        <v>0.354685472353778</v>
+        <v>0.3546854723537781</v>
       </c>
       <c r="G280" t="n">
         <v>66968</v>
@@ -26544,7 +25984,7 @@
         <v>10.59990746047573</v>
       </c>
       <c r="J280" t="n">
-        <v>2.146141140670536</v>
+        <v>2.146141140670535</v>
       </c>
       <c r="K280" t="n">
         <v>73233</v>
@@ -26608,7 +26048,7 @@
         <v>6.318060469808222</v>
       </c>
       <c r="J281" t="n">
-        <v>1.89079619733629</v>
+        <v>1.890796197336291</v>
       </c>
       <c r="K281" t="n">
         <v>4103</v>
@@ -26660,7 +26100,7 @@
         <v>0.321667871880153</v>
       </c>
       <c r="F282" t="n">
-        <v>0.3312283422949549</v>
+        <v>0.331228342294955</v>
       </c>
       <c r="G282" t="n">
         <v>1887</v>
@@ -26788,7 +26228,7 @@
         <v>0.3214737592160181</v>
       </c>
       <c r="F284" t="n">
-        <v>0.3399375209895033</v>
+        <v>0.3399375209895034</v>
       </c>
       <c r="G284" t="n">
         <v>2359</v>
@@ -26977,10 +26417,10 @@
         <v>1</v>
       </c>
       <c r="E287" t="n">
-        <v>0.3211166405134282</v>
+        <v>0.3211166405134283</v>
       </c>
       <c r="F287" t="n">
-        <v>0.3211166405134282</v>
+        <v>0.3211166405134283</v>
       </c>
       <c r="G287" t="n">
         <v>254</v>
@@ -27041,10 +26481,10 @@
         <v>11</v>
       </c>
       <c r="E288" t="n">
-        <v>0.321046976166173</v>
+        <v>0.3210469761661731</v>
       </c>
       <c r="F288" t="n">
-        <v>0.3359631230912986</v>
+        <v>0.3359631230912987</v>
       </c>
       <c r="G288" t="n">
         <v>1688</v>
@@ -27105,7 +26545,7 @@
         <v>2</v>
       </c>
       <c r="E289" t="n">
-        <v>0.3210409320102232</v>
+        <v>0.3210409320102233</v>
       </c>
       <c r="F289" t="n">
         <v>0.3213055618329161</v>
@@ -27233,7 +26673,7 @@
         <v>2</v>
       </c>
       <c r="E291" t="n">
-        <v>0.3206551345760859</v>
+        <v>0.320655134576086</v>
       </c>
       <c r="F291" t="n">
         <v>0.3242809762293826</v>
@@ -27245,7 +26685,7 @@
         <v>161</v>
       </c>
       <c r="I291" t="n">
-        <v>10.93152762946478</v>
+        <v>10.93152762946477</v>
       </c>
       <c r="J291" t="n">
         <v>1.946949602122016</v>
@@ -27364,7 +26804,7 @@
         <v>0.3204368209897947</v>
       </c>
       <c r="F293" t="n">
-        <v>0.3326685353903736</v>
+        <v>0.3326685353903737</v>
       </c>
       <c r="G293" t="n">
         <v>685</v>
@@ -27489,10 +26929,10 @@
         <v>1</v>
       </c>
       <c r="E295" t="n">
-        <v>0.3203380850853581</v>
+        <v>0.3203380850853582</v>
       </c>
       <c r="F295" t="n">
-        <v>0.3203380850853581</v>
+        <v>0.3203380850853582</v>
       </c>
       <c r="G295" t="n">
         <v>259</v>
@@ -27556,7 +26996,7 @@
         <v>0.3202470414526689</v>
       </c>
       <c r="F296" t="n">
-        <v>0.3247176724269185</v>
+        <v>0.3247176724269186</v>
       </c>
       <c r="G296" t="n">
         <v>159</v>
@@ -27684,7 +27124,7 @@
         <v>0.3202320683080685</v>
       </c>
       <c r="F298" t="n">
-        <v>0.3290600334387848</v>
+        <v>0.3290600334387849</v>
       </c>
       <c r="G298" t="n">
         <v>605</v>
@@ -27760,7 +27200,7 @@
         <v>6.155503853201426</v>
       </c>
       <c r="J299" t="n">
-        <v>1.777033492822966</v>
+        <v>1.777033492822967</v>
       </c>
       <c r="K299" t="n">
         <v>503</v>
@@ -28257,10 +27697,10 @@
         <v>1</v>
       </c>
       <c r="E307" t="n">
-        <v>0.3191475100336163</v>
+        <v>0.3191475100336164</v>
       </c>
       <c r="F307" t="n">
-        <v>0.3191475100336163</v>
+        <v>0.3191475100336164</v>
       </c>
       <c r="G307" t="n">
         <v>156</v>
@@ -28424,7 +27864,7 @@
         <v>1</v>
       </c>
       <c r="R309" t="n">
-        <v>38.35649095918368</v>
+        <v>38.35649095918367</v>
       </c>
       <c r="S309" t="n">
         <v>-0.4861343714285714</v>
@@ -28461,7 +27901,7 @@
         <v>391</v>
       </c>
       <c r="I310" t="n">
-        <v>9.275179886400499</v>
+        <v>9.275179886400501</v>
       </c>
       <c r="J310" t="n">
         <v>2.012082228116711</v>
@@ -28470,7 +27910,7 @@
         <v>602</v>
       </c>
       <c r="L310" t="n">
-        <v>0.968516827655492</v>
+        <v>0.9685168276554921</v>
       </c>
       <c r="M310" t="n">
         <v>32708</v>
@@ -28513,10 +27953,10 @@
         <v>12</v>
       </c>
       <c r="E311" t="n">
-        <v>0.3187239765688959</v>
+        <v>0.318723976568896</v>
       </c>
       <c r="F311" t="n">
-        <v>0.3271661386202826</v>
+        <v>0.3271661386202827</v>
       </c>
       <c r="G311" t="n">
         <v>1784</v>
@@ -28644,7 +28084,7 @@
         <v>0.3186458887224272</v>
       </c>
       <c r="F313" t="n">
-        <v>0.3221233235308547</v>
+        <v>0.3221233235308548</v>
       </c>
       <c r="G313" t="n">
         <v>313</v>
@@ -28662,7 +28102,7 @@
         <v>325</v>
       </c>
       <c r="L313" t="n">
-        <v>0.991435799601858</v>
+        <v>0.9914357996018581</v>
       </c>
       <c r="M313" t="n">
         <v>32501</v>
@@ -28784,7 +28224,7 @@
         <v>10.1736516433682</v>
       </c>
       <c r="J315" t="n">
-        <v>1.558938746438746</v>
+        <v>1.558938746438747</v>
       </c>
       <c r="K315" t="n">
         <v>341</v>
@@ -29089,7 +28529,7 @@
         <v>3</v>
       </c>
       <c r="E320" t="n">
-        <v>0.3182549887196785</v>
+        <v>0.3182549887196786</v>
       </c>
       <c r="F320" t="n">
         <v>0.3188216909457059</v>
@@ -29110,7 +28550,7 @@
         <v>672</v>
       </c>
       <c r="L320" t="n">
-        <v>1.267914973797326</v>
+        <v>1.267914973797327</v>
       </c>
       <c r="M320" t="n">
         <v>27491</v>
@@ -29168,7 +28608,7 @@
         <v>10.00600764545793</v>
       </c>
       <c r="J321" t="n">
-        <v>1.890317567736922</v>
+        <v>1.890317567736923</v>
       </c>
       <c r="K321" t="n">
         <v>334</v>
@@ -29284,7 +28724,7 @@
         <v>0.3178081686324966</v>
       </c>
       <c r="F323" t="n">
-        <v>0.344094364382571</v>
+        <v>0.3440943643825711</v>
       </c>
       <c r="G323" t="n">
         <v>1981</v>
@@ -29348,7 +28788,7 @@
         <v>0.3175382503600953</v>
       </c>
       <c r="F324" t="n">
-        <v>0.3233075797288346</v>
+        <v>0.3233075797288347</v>
       </c>
       <c r="G324" t="n">
         <v>410</v>
@@ -29857,7 +29297,7 @@
         <v>4</v>
       </c>
       <c r="E332" t="n">
-        <v>0.3166344380501802</v>
+        <v>0.3166344380501803</v>
       </c>
       <c r="F332" t="n">
         <v>0.3190591922373012</v>
@@ -29872,7 +29312,7 @@
         <v>13.96103243382594</v>
       </c>
       <c r="J332" t="n">
-        <v>1.898077010938698</v>
+        <v>1.898077010938699</v>
       </c>
       <c r="K332" t="n">
         <v>645</v>
@@ -30177,10 +29617,10 @@
         <v>1</v>
       </c>
       <c r="E337" t="n">
-        <v>0.3164440578764887</v>
+        <v>0.3164440578764888</v>
       </c>
       <c r="F337" t="n">
-        <v>0.3164440578764887</v>
+        <v>0.3164440578764888</v>
       </c>
       <c r="G337" t="n">
         <v>40</v>
@@ -30317,7 +29757,7 @@
         <v>1487</v>
       </c>
       <c r="I339" t="n">
-        <v>7.910923727941268</v>
+        <v>7.910923727941269</v>
       </c>
       <c r="J339" t="n">
         <v>1.738632581223976</v>
@@ -30576,7 +30016,7 @@
         <v>12.37696682640618</v>
       </c>
       <c r="J343" t="n">
-        <v>2.039484942171521</v>
+        <v>2.039484942171522</v>
       </c>
       <c r="K343" t="n">
         <v>12258</v>
@@ -30628,7 +30068,7 @@
         <v>0.3157357496315826</v>
       </c>
       <c r="F344" t="n">
-        <v>0.3307535160440208</v>
+        <v>0.3307535160440209</v>
       </c>
       <c r="G344" t="n">
         <v>584</v>
@@ -30646,7 +30086,7 @@
         <v>519</v>
       </c>
       <c r="L344" t="n">
-        <v>0.9028926897068824</v>
+        <v>0.9028926897068823</v>
       </c>
       <c r="M344" t="n">
         <v>29705</v>
@@ -30753,7 +30193,7 @@
         <v>8</v>
       </c>
       <c r="E346" t="n">
-        <v>0.3157004409217342</v>
+        <v>0.3157004409217343</v>
       </c>
       <c r="F346" t="n">
         <v>0.3309952264876523</v>
@@ -30945,10 +30385,10 @@
         <v>1</v>
       </c>
       <c r="E349" t="n">
-        <v>0.3155853613788213</v>
+        <v>0.3155853613788214</v>
       </c>
       <c r="F349" t="n">
-        <v>0.3155853613788213</v>
+        <v>0.3155853613788214</v>
       </c>
       <c r="G349" t="n">
         <v>15</v>
@@ -31329,10 +30769,10 @@
         <v>1</v>
       </c>
       <c r="E355" t="n">
-        <v>0.3150097940746545</v>
+        <v>0.3150097940746546</v>
       </c>
       <c r="F355" t="n">
-        <v>0.3150097940746545</v>
+        <v>0.3150097940746546</v>
       </c>
       <c r="G355" t="n">
         <v>37</v>
@@ -31457,10 +30897,10 @@
         <v>1</v>
       </c>
       <c r="E357" t="n">
-        <v>0.3148460959716987</v>
+        <v>0.3148460959716988</v>
       </c>
       <c r="F357" t="n">
-        <v>0.3148460959716987</v>
+        <v>0.3148460959716988</v>
       </c>
       <c r="G357" t="n">
         <v>163</v>
@@ -31652,7 +31092,7 @@
         <v>0.3147523774388667</v>
       </c>
       <c r="F360" t="n">
-        <v>0.3215192950258321</v>
+        <v>0.3215192950258322</v>
       </c>
       <c r="G360" t="n">
         <v>1155</v>
@@ -31905,10 +31345,10 @@
         <v>1</v>
       </c>
       <c r="E364" t="n">
-        <v>0.3144971705425547</v>
+        <v>0.3144971705425548</v>
       </c>
       <c r="F364" t="n">
-        <v>0.3144971705425547</v>
+        <v>0.3144971705425548</v>
       </c>
       <c r="G364" t="n">
         <v>72</v>
@@ -31969,10 +31409,10 @@
         <v>1</v>
       </c>
       <c r="E365" t="n">
-        <v>0.3144107114596898</v>
+        <v>0.3144107114596899</v>
       </c>
       <c r="F365" t="n">
-        <v>0.3144107114596898</v>
+        <v>0.3144107114596899</v>
       </c>
       <c r="G365" t="n">
         <v>29</v>
@@ -32033,7 +31473,7 @@
         <v>9</v>
       </c>
       <c r="E366" t="n">
-        <v>0.3143448520914907</v>
+        <v>0.3143448520914908</v>
       </c>
       <c r="F366" t="n">
         <v>0.3232056845014462</v>
@@ -32481,10 +31921,10 @@
         <v>1</v>
       </c>
       <c r="E373" t="n">
-        <v>0.312985779224541</v>
+        <v>0.3129857792245411</v>
       </c>
       <c r="F373" t="n">
-        <v>0.312985779224541</v>
+        <v>0.3129857792245411</v>
       </c>
       <c r="G373" t="n">
         <v>153</v>
@@ -32749,7 +32189,7 @@
         <v>150</v>
       </c>
       <c r="I377" t="n">
-        <v>7.00877505238326</v>
+        <v>7.008775052383259</v>
       </c>
       <c r="J377" t="n">
         <v>1.246612466124661</v>
@@ -32865,10 +32305,10 @@
         <v>1</v>
       </c>
       <c r="E379" t="n">
-        <v>0.3120280817996821</v>
+        <v>0.3120280817996822</v>
       </c>
       <c r="F379" t="n">
-        <v>0.3120280817996821</v>
+        <v>0.3120280817996822</v>
       </c>
       <c r="G379" t="n">
         <v>26</v>
@@ -32929,10 +32369,10 @@
         <v>1</v>
       </c>
       <c r="E380" t="n">
-        <v>0.3119869431567872</v>
+        <v>0.3119869431567873</v>
       </c>
       <c r="F380" t="n">
-        <v>0.3119869431567872</v>
+        <v>0.3119869431567873</v>
       </c>
       <c r="G380" t="n">
         <v>104</v>
@@ -32993,7 +32433,7 @@
         <v>2</v>
       </c>
       <c r="E381" t="n">
-        <v>0.3119485255053589</v>
+        <v>0.311948525505359</v>
       </c>
       <c r="F381" t="n">
         <v>0.317922363817449</v>
@@ -33185,7 +32625,7 @@
         <v>2</v>
       </c>
       <c r="E384" t="n">
-        <v>0.3115085337220818</v>
+        <v>0.3115085337220819</v>
       </c>
       <c r="F384" t="n">
         <v>0.3156893620498343</v>
@@ -33249,10 +32689,10 @@
         <v>1</v>
       </c>
       <c r="E385" t="n">
-        <v>0.3113934913705073</v>
+        <v>0.3113934913705074</v>
       </c>
       <c r="F385" t="n">
-        <v>0.3113934913705073</v>
+        <v>0.3113934913705074</v>
       </c>
       <c r="G385" t="n">
         <v>95</v>
@@ -33313,10 +32753,10 @@
         <v>1</v>
       </c>
       <c r="E386" t="n">
-        <v>0.3112667363690339</v>
+        <v>0.311266736369034</v>
       </c>
       <c r="F386" t="n">
-        <v>0.3112667363690339</v>
+        <v>0.311266736369034</v>
       </c>
       <c r="G386" t="n">
         <v>25</v>
@@ -33377,7 +32817,7 @@
         <v>2</v>
       </c>
       <c r="E387" t="n">
-        <v>0.3112113120402724</v>
+        <v>0.3112113120402725</v>
       </c>
       <c r="F387" t="n">
         <v>0.314460858029472</v>
@@ -33441,10 +32881,10 @@
         <v>1</v>
       </c>
       <c r="E388" t="n">
-        <v>0.3111159224342011</v>
+        <v>0.3111159224342012</v>
       </c>
       <c r="F388" t="n">
-        <v>0.3111159224342011</v>
+        <v>0.3111159224342012</v>
       </c>
       <c r="G388" t="n">
         <v>37</v>
@@ -33825,7 +33265,7 @@
         <v>5</v>
       </c>
       <c r="E394" t="n">
-        <v>0.3102056398691096</v>
+        <v>0.3102056398691097</v>
       </c>
       <c r="F394" t="n">
         <v>0.3192455715867416</v>
@@ -33837,7 +33277,7 @@
         <v>618</v>
       </c>
       <c r="I394" t="n">
-        <v>10.05342216980452</v>
+        <v>10.05342216980451</v>
       </c>
       <c r="J394" t="n">
         <v>2.075693360898736</v>
@@ -33892,7 +33332,7 @@
         <v>0.3101660850232988</v>
       </c>
       <c r="F395" t="n">
-        <v>0.3243120795072576</v>
+        <v>0.3243120795072577</v>
       </c>
       <c r="G395" t="n">
         <v>5638</v>
@@ -33968,7 +33408,7 @@
         <v>11.76383295469065</v>
       </c>
       <c r="J396" t="n">
-        <v>1.746942221864823</v>
+        <v>1.746942221864822</v>
       </c>
       <c r="K396" t="n">
         <v>672</v>
@@ -34145,10 +33585,10 @@
         <v>1</v>
       </c>
       <c r="E399" t="n">
-        <v>0.3096426320229223</v>
+        <v>0.3096426320229224</v>
       </c>
       <c r="F399" t="n">
-        <v>0.3096426320229223</v>
+        <v>0.3096426320229224</v>
       </c>
       <c r="G399" t="n">
         <v>50</v>
@@ -34212,7 +33652,7 @@
         <v>0.3094646977424613</v>
       </c>
       <c r="F400" t="n">
-        <v>0.3096960199464252</v>
+        <v>0.3096960199464253</v>
       </c>
       <c r="G400" t="n">
         <v>299</v>
@@ -34273,10 +33713,10 @@
         <v>1</v>
       </c>
       <c r="E401" t="n">
-        <v>0.3094338085819328</v>
+        <v>0.3094338085819329</v>
       </c>
       <c r="F401" t="n">
-        <v>0.3094338085819328</v>
+        <v>0.3094338085819329</v>
       </c>
       <c r="G401" t="n">
         <v>190</v>
@@ -34337,10 +33777,10 @@
         <v>1</v>
       </c>
       <c r="E402" t="n">
-        <v>0.3093870291278734</v>
+        <v>0.3093870291278735</v>
       </c>
       <c r="F402" t="n">
-        <v>0.3093870291278734</v>
+        <v>0.3093870291278735</v>
       </c>
       <c r="G402" t="n">
         <v>133</v>
@@ -34529,7 +33969,7 @@
         <v>18</v>
       </c>
       <c r="E405" t="n">
-        <v>0.3090724413734105</v>
+        <v>0.3090724413734106</v>
       </c>
       <c r="F405" t="n">
         <v>0.3224307257577231</v>
@@ -34593,7 +34033,7 @@
         <v>436</v>
       </c>
       <c r="E406" t="n">
-        <v>0.3090579140518368</v>
+        <v>0.3090579140518369</v>
       </c>
       <c r="F406" t="n">
         <v>0.3444812024480358</v>
@@ -34657,7 +34097,7 @@
         <v>22</v>
       </c>
       <c r="E407" t="n">
-        <v>0.3090535297640085</v>
+        <v>0.3090535297640086</v>
       </c>
       <c r="F407" t="n">
         <v>0.3263443137764212</v>
@@ -34678,7 +34118,7 @@
         <v>3078</v>
       </c>
       <c r="L407" t="n">
-        <v>1.21113253280489</v>
+        <v>1.211132532804891</v>
       </c>
       <c r="M407" t="n">
         <v>30427</v>
@@ -35425,10 +34865,10 @@
         <v>1</v>
       </c>
       <c r="E419" t="n">
-        <v>0.307028722324987</v>
+        <v>0.3070287223249871</v>
       </c>
       <c r="F419" t="n">
-        <v>0.307028722324987</v>
+        <v>0.3070287223249871</v>
       </c>
       <c r="G419" t="n">
         <v>38</v>
@@ -35568,7 +35008,7 @@
         <v>7.913010461386512</v>
       </c>
       <c r="J421" t="n">
-        <v>1.751035196687371</v>
+        <v>1.75103519668737</v>
       </c>
       <c r="K421" t="n">
         <v>381</v>
@@ -35681,7 +35121,7 @@
         <v>14</v>
       </c>
       <c r="E423" t="n">
-        <v>0.3064668388202723</v>
+        <v>0.3064668388202724</v>
       </c>
       <c r="F423" t="n">
         <v>0.3171263849706852</v>
@@ -36004,7 +35444,7 @@
         <v>0.3056068954894542</v>
       </c>
       <c r="F428" t="n">
-        <v>0.3222022697792508</v>
+        <v>0.3222022697792509</v>
       </c>
       <c r="G428" t="n">
         <v>5148</v>
@@ -36065,7 +35505,7 @@
         <v>20</v>
       </c>
       <c r="E429" t="n">
-        <v>0.3055782913036606</v>
+        <v>0.3055782913036607</v>
       </c>
       <c r="F429" t="n">
         <v>0.315835867304829</v>
@@ -36086,7 +35526,7 @@
         <v>3389</v>
       </c>
       <c r="L429" t="n">
-        <v>1.161003006042746</v>
+        <v>1.161003006042747</v>
       </c>
       <c r="M429" t="n">
         <v>29827</v>
@@ -36129,10 +35569,10 @@
         <v>1</v>
       </c>
       <c r="E430" t="n">
-        <v>0.3055777951669587</v>
+        <v>0.3055777951669588</v>
       </c>
       <c r="F430" t="n">
-        <v>0.3055777951669587</v>
+        <v>0.3055777951669588</v>
       </c>
       <c r="G430" t="n">
         <v>210</v>
@@ -36705,10 +36145,10 @@
         <v>1</v>
       </c>
       <c r="E439" t="n">
-        <v>0.3040173742022928</v>
+        <v>0.3040173742022929</v>
       </c>
       <c r="F439" t="n">
-        <v>0.3040173742022928</v>
+        <v>0.3040173742022929</v>
       </c>
       <c r="G439" t="n">
         <v>28</v>
@@ -36772,7 +36212,7 @@
         <v>0.303875080186826</v>
       </c>
       <c r="F440" t="n">
-        <v>0.3107946203529896</v>
+        <v>0.3107946203529897</v>
       </c>
       <c r="G440" t="n">
         <v>1106</v>
@@ -36833,10 +36273,10 @@
         <v>1</v>
       </c>
       <c r="E441" t="n">
-        <v>0.3038322072544597</v>
+        <v>0.3038322072544598</v>
       </c>
       <c r="F441" t="n">
-        <v>0.3038322072544597</v>
+        <v>0.3038322072544598</v>
       </c>
       <c r="G441" t="n">
         <v>94</v>
@@ -36897,7 +36337,7 @@
         <v>24</v>
       </c>
       <c r="E442" t="n">
-        <v>0.3037284871873534</v>
+        <v>0.3037284871873535</v>
       </c>
       <c r="F442" t="n">
         <v>0.3163917054120908</v>
@@ -37601,10 +37041,10 @@
         <v>3</v>
       </c>
       <c r="E453" t="n">
-        <v>0.3011101401417282</v>
+        <v>0.3011101401417283</v>
       </c>
       <c r="F453" t="n">
-        <v>0.3051157463326815</v>
+        <v>0.3051157463326816</v>
       </c>
       <c r="G453" t="n">
         <v>428</v>
@@ -37643,7 +37083,7 @@
         <v>39.53594933333333</v>
       </c>
       <c r="S453" t="n">
-        <v>-0.4131933333333333</v>
+        <v>-0.4131933333333334</v>
       </c>
       <c r="T453" t="n">
         <v>452</v>
@@ -37732,7 +37172,7 @@
         <v>0.3009533206352796</v>
       </c>
       <c r="F455" t="n">
-        <v>0.3100245477052818</v>
+        <v>0.3100245477052819</v>
       </c>
       <c r="G455" t="n">
         <v>1951</v>
@@ -37793,10 +37233,10 @@
         <v>1</v>
       </c>
       <c r="E456" t="n">
-        <v>0.3008142620710641</v>
+        <v>0.3008142620710642</v>
       </c>
       <c r="F456" t="n">
-        <v>0.3008142620710641</v>
+        <v>0.3008142620710642</v>
       </c>
       <c r="G456" t="n">
         <v>75</v>
@@ -38070,7 +37510,7 @@
         <v>10257</v>
       </c>
       <c r="L460" t="n">
-        <v>0.9603380913481584</v>
+        <v>0.9603380913481585</v>
       </c>
       <c r="M460" t="n">
         <v>28193</v>
@@ -38192,7 +37632,7 @@
         <v>11.65582751425326</v>
       </c>
       <c r="J462" t="n">
-        <v>1.740500258576812</v>
+        <v>1.740500258576811</v>
       </c>
       <c r="K462" t="n">
         <v>29207</v>
@@ -38217,7 +37657,7 @@
         <v>42.85095603614458</v>
       </c>
       <c r="S462" t="n">
-        <v>-2.677920487951808</v>
+        <v>-2.677920487951807</v>
       </c>
       <c r="T462" t="n">
         <v>461</v>
@@ -38370,7 +37810,7 @@
         <v>0.2974216980227385</v>
       </c>
       <c r="F465" t="n">
-        <v>0.3087666540190922</v>
+        <v>0.3087666540190923</v>
       </c>
       <c r="G465" t="n">
         <v>433</v>
@@ -38495,7 +37935,7 @@
         <v>164</v>
       </c>
       <c r="E467" t="n">
-        <v>0.2967169242625251</v>
+        <v>0.2967169242625252</v>
       </c>
       <c r="F467" t="n">
         <v>0.3169867543189262</v>
@@ -38623,7 +38063,7 @@
         <v>12</v>
       </c>
       <c r="E469" t="n">
-        <v>0.2942561307048359</v>
+        <v>0.294256130704836</v>
       </c>
       <c r="F469" t="n">
         <v>0.3051684946176933</v>
@@ -38754,7 +38194,7 @@
         <v>0.2939417504730179</v>
       </c>
       <c r="F471" t="n">
-        <v>0.3085524535061474</v>
+        <v>0.3085524535061475</v>
       </c>
       <c r="G471" t="n">
         <v>2799</v>
@@ -38958,7 +38398,7 @@
         <v>12.41265615146908</v>
       </c>
       <c r="J474" t="n">
-        <v>1.756206548892384</v>
+        <v>1.756206548892383</v>
       </c>
       <c r="K474" t="n">
         <v>1791</v>
@@ -39497,7 +38937,7 @@
         <v>35.28889113636364</v>
       </c>
       <c r="S482" t="n">
-        <v>-2.946369295454545</v>
+        <v>-2.946369295454546</v>
       </c>
       <c r="T482" t="n">
         <v>481</v>
@@ -39586,7 +39026,7 @@
         <v>0.2894748958897518</v>
       </c>
       <c r="F484" t="n">
-        <v>0.3350688975420893</v>
+        <v>0.3350688975420894</v>
       </c>
       <c r="G484" t="n">
         <v>34198</v>
@@ -39604,7 +39044,7 @@
         <v>36071</v>
       </c>
       <c r="L484" t="n">
-        <v>1.03688677776142</v>
+        <v>1.036886777761419</v>
       </c>
       <c r="M484" t="n">
         <v>31139</v>
@@ -39650,7 +39090,7 @@
         <v>0.289130782821451</v>
       </c>
       <c r="F485" t="n">
-        <v>0.3153751110729922</v>
+        <v>0.3153751110729923</v>
       </c>
       <c r="G485" t="n">
         <v>35560</v>
@@ -39711,10 +39151,10 @@
         <v>3</v>
       </c>
       <c r="E486" t="n">
-        <v>0.2889505129230268</v>
+        <v>0.2889505129230269</v>
       </c>
       <c r="F486" t="n">
-        <v>0.2985986729281932</v>
+        <v>0.2985986729281933</v>
       </c>
       <c r="G486" t="n">
         <v>598</v>
@@ -39775,7 +39215,7 @@
         <v>84</v>
       </c>
       <c r="E487" t="n">
-        <v>0.2886998744632298</v>
+        <v>0.2886998744632299</v>
       </c>
       <c r="F487" t="n">
         <v>0.315863057153002</v>
@@ -39903,10 +39343,10 @@
         <v>1</v>
       </c>
       <c r="E489" t="n">
-        <v>0.2881091710155672</v>
+        <v>0.2881091710155673</v>
       </c>
       <c r="F489" t="n">
-        <v>0.2881091710155672</v>
+        <v>0.2881091710155673</v>
       </c>
       <c r="G489" t="n">
         <v>22</v>
@@ -40098,7 +39538,7 @@
         <v>0.2865922193769849</v>
       </c>
       <c r="F492" t="n">
-        <v>0.2921104624413645</v>
+        <v>0.2921104624413646</v>
       </c>
       <c r="G492" t="n">
         <v>502</v>
@@ -40287,7 +39727,7 @@
         <v>87</v>
       </c>
       <c r="E495" t="n">
-        <v>0.2856866982292256</v>
+        <v>0.2856866982292257</v>
       </c>
       <c r="F495" t="n">
         <v>0.3081897637275707</v>
@@ -40302,7 +39742,7 @@
         <v>8.024810093925742</v>
       </c>
       <c r="J495" t="n">
-        <v>1.698042052441506</v>
+        <v>1.698042052441507</v>
       </c>
       <c r="K495" t="n">
         <v>11687</v>
@@ -40482,7 +39922,7 @@
         <v>0.2842168595442841</v>
       </c>
       <c r="F498" t="n">
-        <v>0.2920491601937034</v>
+        <v>0.2920491601937035</v>
       </c>
       <c r="G498" t="n">
         <v>2458</v>
@@ -40582,7 +40022,7 @@
         <v>1</v>
       </c>
       <c r="R499" t="n">
-        <v>28.48232125925927</v>
+        <v>28.48232125925926</v>
       </c>
       <c r="S499" t="n">
         <v>-16.3161704537037</v>
@@ -40607,10 +40047,10 @@
         <v>253</v>
       </c>
       <c r="E500" t="n">
-        <v>0.2840728243335207</v>
+        <v>0.2840728243335208</v>
       </c>
       <c r="F500" t="n">
-        <v>0.3070093945519804</v>
+        <v>0.3070093945519805</v>
       </c>
       <c r="G500" t="n">
         <v>30848</v>
@@ -41553,7 +40993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41579,6 +41019,16 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>pension</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>precio_m2</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>fofm_medio</t>
         </is>
       </c>
@@ -41599,6 +41049,12 @@
         <v>19064.73</v>
       </c>
       <c r="E2" t="n">
+        <v>1463.6</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2002.33</v>
+      </c>
+      <c r="G2" t="n">
         <v>0.28</v>
       </c>
     </row>
@@ -41618,6 +41074,12 @@
         <v>103063.75</v>
       </c>
       <c r="E3" t="n">
+        <v>1479.83</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2995.62</v>
+      </c>
+      <c r="G3" t="n">
         <v>0.35</v>
       </c>
     </row>
@@ -41637,6 +41099,12 @@
         <v>5158.04</v>
       </c>
       <c r="E4" t="n">
+        <v>1363.6</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2016.9</v>
+      </c>
+      <c r="G4" t="n">
         <v>0.27</v>
       </c>
     </row>
@@ -41656,6 +41124,12 @@
         <v>4997.25</v>
       </c>
       <c r="E5" t="n">
+        <v>1818.15</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4757.9</v>
+      </c>
+      <c r="G5" t="n">
         <v>0.51</v>
       </c>
     </row>
@@ -41705,7 +41179,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Gráfico de barras con los 4 perfiles estratégicos — meter en slides</t>
+          <t>Gráfico de barras con los 4 perfiles estratégicos</t>
         </is>
       </c>
     </row>
@@ -41717,7 +41191,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ranking visual del top 20 municipios — meter en slides</t>
+          <t>Ranking visual del top 20 municipios</t>
         </is>
       </c>
     </row>
@@ -41729,7 +41203,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Scatter solvencia vs mercado — meter en slides</t>
+          <t>Scatter solvencia vs tamaño de mercado</t>
         </is>
       </c>
     </row>

</xml_diff>